<commit_message>
for mr bakaev #2
</commit_message>
<xml_diff>
--- a/library/power_supplies.xlsx
+++ b/library/power_supplies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CAF751-9357-4B3F-86B0-152059D1F1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D825D43-9F90-4DD1-8CAE-49BC58B2B8AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="223">
   <si>
     <t>Part Number</t>
   </si>
@@ -813,6 +813,15 @@
   </si>
   <si>
     <t>бКО.347.098-11 ТУ</t>
+  </si>
+  <si>
+    <t>TO-263-3</t>
+  </si>
+  <si>
+    <t>LM1117SX-5.0</t>
+  </si>
+  <si>
+    <t>LM1117SX-5.0 TO-263-3</t>
   </si>
 </sst>
 </file>
@@ -1926,7 +1935,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A36817BF-F161-418A-9B8F-87A18459EBCD}">
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20.5703125" customWidth="1"/>
@@ -2743,6 +2752,29 @@
       </c>
       <c r="H35" t="s">
         <v>219</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
+        <v>221</v>
+      </c>
+      <c r="B36" t="s">
+        <v>220</v>
+      </c>
+      <c r="C36" t="s">
+        <v>222</v>
+      </c>
+      <c r="D36" t="s">
+        <v>221</v>
+      </c>
+      <c r="E36" t="s">
+        <v>40</v>
+      </c>
+      <c r="F36" t="s">
+        <v>220</v>
+      </c>
+      <c r="G36" t="s">
+        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BLET, BAKAINIY + misc
</commit_message>
<xml_diff>
--- a/library/power_supplies.xlsx
+++ b/library/power_supplies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitProjects\elem_altium_db2\library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB42A13D-5878-4218-AA82-B873CCA68BFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771EEA85-7313-4C50-AFF5-4F7CE3775640}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{EE2E7F00-6B54-4C0B-98D7-835E87062BAF}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="246">
   <si>
     <t>Part Number</t>
   </si>
@@ -919,6 +919,9 @@
   </si>
   <si>
     <t>LT3757EMSE 10-MSOP</t>
+  </si>
+  <si>
+    <t>10-MSOP (PAD)</t>
   </si>
 </sst>
 </file>
@@ -2027,7 +2030,7 @@
         <v>241</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>156</v>

</xml_diff>